<commit_message>
walk through the last three figures; every step is now a Quarto walkthrough
</commit_message>
<xml_diff>
--- a/05_Figures/Continuous/F1_Overview/c_data/f1_overview.xlsx
+++ b/05_Figures/Continuous/F1_Overview/c_data/f1_overview.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5669" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5699" uniqueCount="415">
   <si>
     <t>sheet</t>
   </si>
@@ -795,13 +795,13 @@
     <t>04_Continuous_no_group/01_Trait_Associations/01_Proteins/c_data/protein_trait_associations.xlsx</t>
   </si>
   <si>
-    <t>400e71a7f9b28b71965d7d0a160d06c9</t>
+    <t>4c94a3c340f52458c17e5a5394bde99d</t>
   </si>
   <si>
     <t>04_Continuous_no_group/01_Trait_Associations/02_Sets/c_data/set_trait_associations.xlsx</t>
   </si>
   <si>
-    <t>3d21c84292f410b6f34c484bd5074e96</t>
+    <t>7f37044c17c08e80c99d1556b6aa9911</t>
   </si>
   <si>
     <t>modules</t>
@@ -810,7 +810,7 @@
     <t>04_Continuous_no_group/01_Trait_Associations/03_Modules/c_data/module_trait_associations.xlsx</t>
   </si>
   <si>
-    <t>ff084ce743cbe0bc8a39fddd8f920530</t>
+    <t>0d7339fe075482c3e9b058848e322883</t>
   </si>
   <si>
     <t>pathways</t>
@@ -819,7 +819,7 @@
     <t>04_Continuous_no_group/02_Trait_Pathways/c_data/trait_pathways.xlsx</t>
   </si>
   <si>
-    <t>37b270811c8ae46c10a723e86f5256e5</t>
+    <t>dcf258c971d240ae00d1de43e40aec20</t>
   </si>
   <si>
     <t>gene_sets</t>
@@ -834,7 +834,7 @@
     <t>04_Continuous_no_group/03_Profile_Clusters/c_data/profile_clusters.xlsx</t>
   </si>
   <si>
-    <t>e27701d11c4ee900dd3353dcc577a065</t>
+    <t>9a237a2de34c62ef092affa6e6f7adea</t>
   </si>
   <si>
     <t>corrected</t>
@@ -849,7 +849,7 @@
     <t>phenotype</t>
   </si>
   <si>
-    <t>00_Input/phenotype.csv</t>
+    <t>00_Setup/Input/phenotype.csv</t>
   </si>
   <si>
     <t>5a1989db406daa0b70189a9f0df52cf3</t>
@@ -957,10 +957,22 @@
     <t>1.2.1</t>
   </si>
   <si>
+    <t>evaluate</t>
+  </si>
+  <si>
+    <t>1.0.5</t>
+  </si>
+  <si>
     <t>farver</t>
   </si>
   <si>
     <t>2.1.2</t>
+  </si>
+  <si>
+    <t>fastmap</t>
+  </si>
+  <si>
+    <t>1.2.0</t>
   </si>
   <si>
     <t>foreach</t>
@@ -1014,6 +1026,18 @@
     <t>1.1.4</t>
   </si>
   <si>
+    <t>htmltools</t>
+  </si>
+  <si>
+    <t>0.5.9</t>
+  </si>
+  <si>
+    <t>htmlwidgets</t>
+  </si>
+  <si>
+    <t>1.6.4</t>
+  </si>
+  <si>
     <t>IRanges</t>
   </si>
   <si>
@@ -1026,6 +1050,18 @@
     <t>1.0.14</t>
   </si>
   <si>
+    <t>jsonlite</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
+  </si>
+  <si>
+    <t>knitr</t>
+  </si>
+  <si>
+    <t>1.51</t>
+  </si>
+  <si>
     <t>labeling</t>
   </si>
   <si>
@@ -1033,9 +1069,6 @@
   </si>
   <si>
     <t>lifecycle</t>
-  </si>
-  <si>
-    <t>1.0.5</t>
   </si>
   <si>
     <t>magrittr</t>
@@ -1048,6 +1081,12 @@
   </si>
   <si>
     <t>1.5.0</t>
+  </si>
+  <si>
+    <t>otel</t>
+  </si>
+  <si>
+    <t>0.2.0</t>
   </si>
   <si>
     <t>patchwork</t>
@@ -1123,6 +1162,12 @@
   </si>
   <si>
     <t>CRAN (R 4.6.1)</t>
+  </si>
+  <si>
+    <t>rmarkdown</t>
+  </si>
+  <si>
+    <t>2.31</t>
   </si>
   <si>
     <t>rprojroot</t>
@@ -1210,6 +1255,18 @@
   </si>
   <si>
     <t>3.0.2</t>
+  </si>
+  <si>
+    <t>xfun</t>
+  </si>
+  <si>
+    <t>0.57</t>
+  </si>
+  <si>
+    <t>yaml</t>
+  </si>
+  <si>
+    <t>2.3.12</t>
   </si>
 </sst>
 </file>
@@ -43682,7 +43739,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -43932,7 +43989,7 @@
         <v>321</v>
       </c>
       <c r="B23" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="C23" t="s">
         <v>282</v>
@@ -43940,10 +43997,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B24" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C24" t="s">
         <v>282</v>
@@ -43951,10 +44008,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B25" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="C25" t="s">
         <v>282</v>
@@ -43990,7 +44047,7 @@
         <v>331</v>
       </c>
       <c r="C28" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -44034,7 +44091,7 @@
         <v>339</v>
       </c>
       <c r="C32" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -44086,7 +44143,7 @@
         <v>348</v>
       </c>
       <c r="B37" t="s">
-        <v>349</v>
+        <v>312</v>
       </c>
       <c r="C37" t="s">
         <v>282</v>
@@ -44094,10 +44151,10 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
+        <v>349</v>
+      </c>
+      <c r="B38" t="s">
         <v>350</v>
-      </c>
-      <c r="B38" t="s">
-        <v>351</v>
       </c>
       <c r="C38" t="s">
         <v>282</v>
@@ -44105,10 +44162,10 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
+        <v>351</v>
+      </c>
+      <c r="B39" t="s">
         <v>352</v>
-      </c>
-      <c r="B39" t="s">
-        <v>353</v>
       </c>
       <c r="C39" t="s">
         <v>282</v>
@@ -44116,10 +44173,10 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
+        <v>353</v>
+      </c>
+      <c r="B40" t="s">
         <v>354</v>
-      </c>
-      <c r="B40" t="s">
-        <v>355</v>
       </c>
       <c r="C40" t="s">
         <v>282</v>
@@ -44127,10 +44184,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
+        <v>355</v>
+      </c>
+      <c r="B41" t="s">
         <v>356</v>
-      </c>
-      <c r="B41" t="s">
-        <v>357</v>
       </c>
       <c r="C41" t="s">
         <v>282</v>
@@ -44138,10 +44195,10 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
+        <v>357</v>
+      </c>
+      <c r="B42" t="s">
         <v>358</v>
-      </c>
-      <c r="B42" t="s">
-        <v>359</v>
       </c>
       <c r="C42" t="s">
         <v>282</v>
@@ -44149,10 +44206,10 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
+        <v>359</v>
+      </c>
+      <c r="B43" t="s">
         <v>360</v>
-      </c>
-      <c r="B43" t="s">
-        <v>361</v>
       </c>
       <c r="C43" t="s">
         <v>282</v>
@@ -44160,10 +44217,10 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
+        <v>361</v>
+      </c>
+      <c r="B44" t="s">
         <v>362</v>
-      </c>
-      <c r="B44" t="s">
-        <v>363</v>
       </c>
       <c r="C44" t="s">
         <v>282</v>
@@ -44171,21 +44228,21 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
+        <v>363</v>
+      </c>
+      <c r="B45" t="s">
         <v>364</v>
       </c>
-      <c r="B45" t="s">
-        <v>365</v>
-      </c>
       <c r="C45" t="s">
-        <v>366</v>
+        <v>282</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B46" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C46" t="s">
         <v>282</v>
@@ -44193,21 +44250,21 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B47" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C47" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B48" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C48" t="s">
         <v>282</v>
@@ -44215,10 +44272,10 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B49" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C49" t="s">
         <v>282</v>
@@ -44226,10 +44283,10 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B50" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C50" t="s">
         <v>282</v>
@@ -44237,10 +44294,10 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B51" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C51" t="s">
         <v>282</v>
@@ -44248,21 +44305,21 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
+        <v>377</v>
+      </c>
+      <c r="B52" t="s">
+        <v>378</v>
+      </c>
+      <c r="C52" t="s">
         <v>379</v>
-      </c>
-      <c r="B52" t="s">
-        <v>380</v>
-      </c>
-      <c r="C52" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
+        <v>380</v>
+      </c>
+      <c r="B53" t="s">
         <v>381</v>
-      </c>
-      <c r="B53" t="s">
-        <v>382</v>
       </c>
       <c r="C53" t="s">
         <v>282</v>
@@ -44270,10 +44327,10 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
+        <v>382</v>
+      </c>
+      <c r="B54" t="s">
         <v>383</v>
-      </c>
-      <c r="B54" t="s">
-        <v>384</v>
       </c>
       <c r="C54" t="s">
         <v>282</v>
@@ -44281,13 +44338,13 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
+        <v>384</v>
+      </c>
+      <c r="B55" t="s">
         <v>385</v>
       </c>
-      <c r="B55" t="s">
-        <v>343</v>
-      </c>
       <c r="C55" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -44295,7 +44352,7 @@
         <v>386</v>
       </c>
       <c r="B56" t="s">
-        <v>310</v>
+        <v>387</v>
       </c>
       <c r="C56" t="s">
         <v>282</v>
@@ -44303,10 +44360,10 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B57" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C57" t="s">
         <v>282</v>
@@ -44314,10 +44371,10 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B58" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C58" t="s">
         <v>282</v>
@@ -44325,10 +44382,10 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B59" t="s">
-        <v>335</v>
+        <v>393</v>
       </c>
       <c r="C59" t="s">
         <v>282</v>
@@ -44336,10 +44393,10 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B60" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="C60" t="s">
         <v>282</v>
@@ -44347,12 +44404,122 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B61" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="C61" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
+        <v>398</v>
+      </c>
+      <c r="B62" t="s">
+        <v>399</v>
+      </c>
+      <c r="C62" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
+        <v>400</v>
+      </c>
+      <c r="B63" t="s">
+        <v>356</v>
+      </c>
+      <c r="C63" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" t="s">
+        <v>401</v>
+      </c>
+      <c r="B64" t="s">
+        <v>310</v>
+      </c>
+      <c r="C64" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" t="s">
+        <v>402</v>
+      </c>
+      <c r="B65" t="s">
+        <v>403</v>
+      </c>
+      <c r="C65" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" t="s">
+        <v>404</v>
+      </c>
+      <c r="B66" t="s">
+        <v>405</v>
+      </c>
+      <c r="C66" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" t="s">
+        <v>406</v>
+      </c>
+      <c r="B67" t="s">
+        <v>347</v>
+      </c>
+      <c r="C67" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" t="s">
+        <v>407</v>
+      </c>
+      <c r="B68" t="s">
+        <v>408</v>
+      </c>
+      <c r="C68" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
+        <v>409</v>
+      </c>
+      <c r="B69" t="s">
+        <v>410</v>
+      </c>
+      <c r="C69" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" t="s">
+        <v>411</v>
+      </c>
+      <c r="B70" t="s">
+        <v>412</v>
+      </c>
+      <c r="C70" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" t="s">
+        <v>413</v>
+      </c>
+      <c r="B71" t="s">
+        <v>414</v>
+      </c>
+      <c r="C71" t="s">
         <v>282</v>
       </c>
     </row>

</xml_diff>

<commit_message>
write each comparison and figure once, and let every grouping run it
</commit_message>
<xml_diff>
--- a/05_Figures/Continuous/F1_Overview/c_data/f1_overview.xlsx
+++ b/05_Figures/Continuous/F1_Overview/c_data/f1_overview.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5699" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5672" uniqueCount="398">
   <si>
     <t>sheet</t>
   </si>
@@ -957,22 +957,10 @@
     <t>1.2.1</t>
   </si>
   <si>
-    <t>evaluate</t>
-  </si>
-  <si>
-    <t>1.0.5</t>
-  </si>
-  <si>
     <t>farver</t>
   </si>
   <si>
     <t>2.1.2</t>
-  </si>
-  <si>
-    <t>fastmap</t>
-  </si>
-  <si>
-    <t>1.2.0</t>
   </si>
   <si>
     <t>foreach</t>
@@ -1026,18 +1014,6 @@
     <t>1.1.4</t>
   </si>
   <si>
-    <t>htmltools</t>
-  </si>
-  <si>
-    <t>0.5.9</t>
-  </si>
-  <si>
-    <t>htmlwidgets</t>
-  </si>
-  <si>
-    <t>1.6.4</t>
-  </si>
-  <si>
     <t>IRanges</t>
   </si>
   <si>
@@ -1050,18 +1026,6 @@
     <t>1.0.14</t>
   </si>
   <si>
-    <t>jsonlite</t>
-  </si>
-  <si>
-    <t>2.0.0</t>
-  </si>
-  <si>
-    <t>knitr</t>
-  </si>
-  <si>
-    <t>1.51</t>
-  </si>
-  <si>
     <t>labeling</t>
   </si>
   <si>
@@ -1069,6 +1033,9 @@
   </si>
   <si>
     <t>lifecycle</t>
+  </si>
+  <si>
+    <t>1.0.5</t>
   </si>
   <si>
     <t>magrittr</t>
@@ -1081,12 +1048,6 @@
   </si>
   <si>
     <t>1.5.0</t>
-  </si>
-  <si>
-    <t>otel</t>
-  </si>
-  <si>
-    <t>0.2.0</t>
   </si>
   <si>
     <t>patchwork</t>
@@ -1162,12 +1123,6 @@
   </si>
   <si>
     <t>CRAN (R 4.6.1)</t>
-  </si>
-  <si>
-    <t>rmarkdown</t>
-  </si>
-  <si>
-    <t>2.31</t>
   </si>
   <si>
     <t>rprojroot</t>
@@ -1255,12 +1210,6 @@
   </si>
   <si>
     <t>3.0.2</t>
-  </si>
-  <si>
-    <t>xfun</t>
-  </si>
-  <si>
-    <t>0.57</t>
   </si>
   <si>
     <t>yaml</t>
@@ -43739,7 +43688,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -43989,7 +43938,7 @@
         <v>321</v>
       </c>
       <c r="B23" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="C23" t="s">
         <v>282</v>
@@ -43997,10 +43946,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
+        <v>322</v>
+      </c>
+      <c r="B24" t="s">
         <v>323</v>
-      </c>
-      <c r="B24" t="s">
-        <v>324</v>
       </c>
       <c r="C24" t="s">
         <v>282</v>
@@ -44008,10 +43957,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
+        <v>324</v>
+      </c>
+      <c r="B25" t="s">
         <v>325</v>
-      </c>
-      <c r="B25" t="s">
-        <v>320</v>
       </c>
       <c r="C25" t="s">
         <v>282</v>
@@ -44047,7 +43996,7 @@
         <v>331</v>
       </c>
       <c r="C28" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -44091,7 +44040,7 @@
         <v>339</v>
       </c>
       <c r="C32" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -44143,7 +44092,7 @@
         <v>348</v>
       </c>
       <c r="B37" t="s">
-        <v>312</v>
+        <v>349</v>
       </c>
       <c r="C37" t="s">
         <v>282</v>
@@ -44151,10 +44100,10 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B38" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C38" t="s">
         <v>282</v>
@@ -44162,10 +44111,10 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B39" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C39" t="s">
         <v>282</v>
@@ -44173,10 +44122,10 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B40" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C40" t="s">
         <v>282</v>
@@ -44184,10 +44133,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B41" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C41" t="s">
         <v>282</v>
@@ -44195,10 +44144,10 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B42" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C42" t="s">
         <v>282</v>
@@ -44206,10 +44155,10 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B43" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C43" t="s">
         <v>282</v>
@@ -44217,10 +44166,10 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B44" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C44" t="s">
         <v>282</v>
@@ -44228,21 +44177,21 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B45" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C45" t="s">
-        <v>282</v>
+        <v>366</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B46" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="C46" t="s">
         <v>282</v>
@@ -44250,21 +44199,21 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B47" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C47" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B48" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="C48" t="s">
         <v>282</v>
@@ -44272,10 +44221,10 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B49" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="C49" t="s">
         <v>282</v>
@@ -44283,10 +44232,10 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B50" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="C50" t="s">
         <v>282</v>
@@ -44294,10 +44243,10 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B51" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C51" t="s">
         <v>282</v>
@@ -44305,21 +44254,21 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B52" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="C52" t="s">
-        <v>379</v>
+        <v>282</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B53" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C53" t="s">
         <v>282</v>
@@ -44327,10 +44276,10 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B54" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C54" t="s">
         <v>282</v>
@@ -44338,13 +44287,13 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B55" t="s">
-        <v>385</v>
+        <v>343</v>
       </c>
       <c r="C55" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -44352,7 +44301,7 @@
         <v>386</v>
       </c>
       <c r="B56" t="s">
-        <v>387</v>
+        <v>310</v>
       </c>
       <c r="C56" t="s">
         <v>282</v>
@@ -44360,10 +44309,10 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
+        <v>387</v>
+      </c>
+      <c r="B57" t="s">
         <v>388</v>
-      </c>
-      <c r="B57" t="s">
-        <v>389</v>
       </c>
       <c r="C57" t="s">
         <v>282</v>
@@ -44371,10 +44320,10 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
+        <v>389</v>
+      </c>
+      <c r="B58" t="s">
         <v>390</v>
-      </c>
-      <c r="B58" t="s">
-        <v>391</v>
       </c>
       <c r="C58" t="s">
         <v>282</v>
@@ -44382,10 +44331,10 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B59" t="s">
-        <v>393</v>
+        <v>335</v>
       </c>
       <c r="C59" t="s">
         <v>282</v>
@@ -44393,10 +44342,10 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B60" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C60" t="s">
         <v>282</v>
@@ -44404,10 +44353,10 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B61" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C61" t="s">
         <v>282</v>
@@ -44415,111 +44364,12 @@
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B62" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C62" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3">
-      <c r="A63" t="s">
-        <v>400</v>
-      </c>
-      <c r="B63" t="s">
-        <v>356</v>
-      </c>
-      <c r="C63" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3">
-      <c r="A64" t="s">
-        <v>401</v>
-      </c>
-      <c r="B64" t="s">
-        <v>310</v>
-      </c>
-      <c r="C64" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3">
-      <c r="A65" t="s">
-        <v>402</v>
-      </c>
-      <c r="B65" t="s">
-        <v>403</v>
-      </c>
-      <c r="C65" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3">
-      <c r="A66" t="s">
-        <v>404</v>
-      </c>
-      <c r="B66" t="s">
-        <v>405</v>
-      </c>
-      <c r="C66" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3">
-      <c r="A67" t="s">
-        <v>406</v>
-      </c>
-      <c r="B67" t="s">
-        <v>347</v>
-      </c>
-      <c r="C67" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3">
-      <c r="A68" t="s">
-        <v>407</v>
-      </c>
-      <c r="B68" t="s">
-        <v>408</v>
-      </c>
-      <c r="C68" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3">
-      <c r="A69" t="s">
-        <v>409</v>
-      </c>
-      <c r="B69" t="s">
-        <v>410</v>
-      </c>
-      <c r="C69" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3">
-      <c r="A70" t="s">
-        <v>411</v>
-      </c>
-      <c r="B70" t="s">
-        <v>412</v>
-      </c>
-      <c r="C70" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3">
-      <c r="A71" t="s">
-        <v>413</v>
-      </c>
-      <c r="B71" t="s">
-        <v>414</v>
-      </c>
-      <c r="C71" t="s">
         <v>282</v>
       </c>
     </row>

</xml_diff>